<commit_message>
La entidad pasa a llamarse publicación y el evento que la crea, publicar: sustantivo para la entidad y verbo para el evento, así no se confunden. Cascada queda para el árbol de reenvíos de una publicación, que es lo que mide el dataset. De paso, la tasa de llegadas queda en semillas por hora (0,51 a las 3, 1,62 a las 17) en vez de las cuentas por franja.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelo-de-datos.xlsx
+++ b/modelo-de-datos.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -648,178 +648,190 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Nombres</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>25/9/2026. Todo sale de muestra_cascadas_REDBAIRES.csv sin las 132 filas duplicadas y de parametros_y_costos.csv.</t>
+          <t>La entidad es la publicación (la pieza original, message_id). Publicar es el evento que la crea. Cascada es el árbol de reenvíos de una publicación, como en el dataset.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Base de las medias</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Las medias de hijos (R) excluyen las 14 cascadas cortadas en 500 eventos (D14), así que algunas difieren un poco de las del README.</t>
+          <t>25/9/2026. Todo sale de muestra_cascadas_REDBAIRES.csv sin las 132 filas duplicadas y de parametros_y_costos.csv.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Colores</t>
+          <t>Base de las medias</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Azul: dato medido o del CSV, cargado a mano. Negro: fórmula. Verde: fórmula que trae un valor de otra hoja. Amarillo: para completar por el grupo.</t>
+          <t>Las medias de hijos (R) excluyen las 14 cascadas cortadas en 500 eventos (D14), así que algunas difieren un poco de las del README.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Modelo de datos</t>
+          <t>Colores</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>La tabla con el formato de la clase 06: variable, U.M., valor, tipo de función, parámetros y relación. Una fila por elemento del modelo conceptual.</t>
+          <t>Azul: dato medido o del CSV, cargado a mano. Negro: fórmula. Verde: fórmula que trae un valor de otra hoja. Amarillo: para completar por el grupo.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Parámetros CSV</t>
+          <t>Modelo de datos</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>parametros_y_costos.csv tal cual, con valor base y rango.</t>
+          <t>La tabla con el formato de la clase 06: variable, U.M., valor, tipo de función, parámetros y relación. Una fila por elemento del modelo conceptual.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Llegadas</t>
+          <t>Parámetros CSV</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Semillas por hora del día y por día de la semana, y la tasa por hora que sale de ahí.</t>
+          <t>parametros_y_costos.csv tal cual, con valor base y rango.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Tipos de cuenta</t>
+          <t>Llegadas</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Mezcla de tipos en semillas y en reenvíos, hijos medios (R) y seguidores por tipo.</t>
+          <t>Semillas por hora del día y por día de la semana, y la tasa por hora que sale de ahí.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Generaciones</t>
+          <t>Tipos de cuenta</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Hijos medios por generación: el decaimiento (D18).</t>
+          <t>Mezcla de tipos en semillas y en reenvíos, hijos medios (R) y seguidores por tipo.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Marca</t>
+          <t>Generaciones</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Probabilidad de que Centinela marque, por tema y quintil de toxicidad.</t>
+          <t>Hijos medios por generación: el decaimiento (D18).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Ajuste D19</t>
+          <t>Marca</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Ajuste de distribuciones al tiempo entre generaciones.</t>
+          <t>Probabilidad de que Centinela marque, por tema y quintil de toxicidad.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Validación</t>
+          <t>Ajuste D19</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Los números que el simulador tiene que reproducir.</t>
+          <t>Ajuste de distribuciones al tiempo entre generaciones.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>A priori</t>
+          <t>Validación</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Cuentas sin simular: tamaño esperado, ocupación del moderador y tipo de cambio. Son fórmulas sobre las otras hojas.</t>
+          <t>Los números que el simulador tiene que reproducir.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Diccionario</t>
+          <t>A priori</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Qué es cada columna de la muestra y cómo lo sabemos.</t>
+          <t>Cuentas sin simular: tamaño esperado, ocupación del moderador y tipo de cambio. Son fórmulas sobre las otras hojas.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Limpieza</t>
+          <t>Diccionario</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Lo sucio de la muestra.</t>
+          <t>Qué es cada columna de la muestra y cómo lo sabemos.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Limpieza</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Lo sucio de la muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Decisiones</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>D1 a D20, como en el README y el artifact. La columna amarilla es para lo que elija el grupo.</t>
         </is>
@@ -1371,7 +1383,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>cascada a la que pertenece</t>
+          <t>cascada: el árbol de reenvíos de una publicación</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -1393,17 +1405,17 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>pieza de contenido</t>
+          <t>la publicación: pieza de contenido original, una por cascada</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>clave</t>
+          <t>clave; 1 a 1 con cascade_id</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>sin uso definido</t>
+          <t>identifica a la entidad</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1427,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>marca el evento original</t>
+          <t>marca la publicación original</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -1425,7 +1437,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>llegadas y su tasa horaria</t>
+          <t>el evento publicar y su tasa horaria</t>
         </is>
       </c>
     </row>
@@ -2324,12 +2336,12 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>la cascada · un lote por generación · el reenvío</t>
+          <t>la publicación · un lote por generación · el reenvío</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>la cascada (DECIDIDA 22/9)</t>
+          <t>la publicación (DECIDIDA 22/9; el nombre, 25/9)</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -2339,7 +2351,7 @@
       </c>
       <c r="F4" s="36" t="inlineStr">
         <is>
-          <t>la cascada</t>
+          <t>la publicación</t>
         </is>
       </c>
     </row>
@@ -2440,12 +2452,12 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>ocupación (obligatoria) · largo de la cola · cascadas vivas e ítems en revisión · R efectivo</t>
+          <t>ocupación (obligatoria) · largo de la cola · publicaciones vivas e ítems en revisión · R efectivo</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>ocupación + cola + cascadas vivas</t>
+          <t>ocupación + cola + publicaciones vivas</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -2711,7 +2723,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>¿Cómo llegan los rumores?</t>
+          <t>¿Cada cuánto ocurre publicar?</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -2960,17 +2972,17 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Evento</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Llegada de rumores</t>
+          <t>Publicar</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>tiempo entre semillas</t>
+          <t>llega un rumor nuevo: crea la publicación. Tiempo entre semillas</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -3002,7 +3014,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Atributo</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -3012,7 +3024,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>con qué cuenta arranca la cascada</t>
+          <t>con qué cuenta se publica</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -4615,7 +4627,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Llegadas de rumores (semillas)</t>
+          <t>Publicar: llegadas de rumores (semillas)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
El diccionario del Excel documenta cada columna del dataset con tipo, rango, faltantes, suciedad, verificación y la decisión que alimenta. De paso se corrigen números del README y de la hoja Limpieza que se habían medido con los duplicados adentro o con las cascadas cortadas, y se separan los 39 tiempos negativos de los 22 hijos que quedan antes del padre por las fechas de 2099.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelo-de-datos.xlsx
+++ b/modelo-de-datos.xlsx
@@ -104,7 +104,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -117,11 +117,25 @@
         <color rgb="00CFD7E1"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -249,6 +263,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -809,7 +838,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Qué es cada columna de la muestra y cómo lo sabemos.</t>
+          <t>Qué es cada columna de la muestra y cómo lo sabemos. Ampliado el 29/9/2026: tipo, unidad, rango, faltantes, suciedad, relaciones, uso y decisión de cada columna.</t>
         </is>
       </c>
     </row>
@@ -1308,13 +1337,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:M33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1327,11 +1365,11 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>RedBaires perdió la documentación de los campos: reconstruirla es parte de la nota.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>RedBaires perdió la documentación de los campos: reconstruirla es parte de la nota. Los números son de las 66.021 filas que quedan sin los 132 duplicados, antes de cualquier otra limpieza, salvo donde se aclara. En azul, lo medido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Columna</t>
@@ -1344,672 +1382,1947 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Cómo lo sabemos</t>
+          <t>Tipo de dato</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Valores / rango</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Faltantes</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>% faltante</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Suciedad detectada y qué hacemos</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Cómo lo sabemos / verificación</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Relación con otras columnas</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
           <t>Uso en el modelo</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="35" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Ejemplo de valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
+      <c r="A4" s="47" t="inlineStr">
         <is>
           <t>event_id</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>identificador del evento</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>clave</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>no entra</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="35" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>Identificador del evento. Cada fila del export es un evento: la publicación original o uno de sus reenvíos. Es la clave de la tabla.</t>
+        </is>
+      </c>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>texto (identificador)</t>
+        </is>
+      </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="49" t="inlineStr">
+        <is>
+          <t>66.021 valores distintos, de la forma E + 7 dígitos (E0000001 a E0066021)</t>
+        </is>
+      </c>
+      <c r="F4" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="48" t="inlineStr">
+        <is>
+          <t>Las 132 filas duplicadas repiten la fila entera, event_id incluido. Se sacan antes de medir y la clave queda única.</t>
+        </is>
+      </c>
+      <c r="I4" s="48" t="inlineStr">
+        <is>
+          <t>Es clave: después de sacar los duplicados cada valor aparece una sola vez.</t>
+        </is>
+      </c>
+      <c r="J4" s="48" t="inlineStr">
+        <is>
+          <t>parent_event_id apunta a un event_id. No hay padres fuera de la muestra: los 61.021 padres existen como event_id.</t>
+        </is>
+      </c>
+      <c r="K4" s="48" t="inlineStr">
+        <is>
+          <t>No entra al modelo; sirve para reconstruir el árbol.</t>
+        </is>
+      </c>
+      <c r="L4" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M4" s="49" t="inlineStr">
+        <is>
+          <t>E0000001</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>cascade_id</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>cascada: el árbol de reenvíos de una publicación</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>clave</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>unidad de validación</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="35" t="inlineStr">
+      <c r="B5" s="48" t="inlineStr">
+        <is>
+          <t>Identificador de la cascada: el árbol de reenvíos que sale de una publicación. Todas las filas de un mismo árbol comparten el valor.</t>
+        </is>
+      </c>
+      <c r="C5" s="48" t="inlineStr">
+        <is>
+          <t>texto (identificador)</t>
+        </is>
+      </c>
+      <c r="D5" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="49" t="inlineStr">
+        <is>
+          <t>5.000 cascadas. Eventos por cascada: mín 1 · p10 1 · mediana 2 · media 13,2 · p90 29 · máx 500. p99 188. 2.019 cascadas (40 %) tienen un solo evento</t>
+        </is>
+      </c>
+      <c r="F5" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>14 cascadas tienen exactamente 500 eventos, todas del sufijo C2: el export corta ahí y la cola está censurada. Se sacan para medir R y la simulación también corta en 500 al validar (D14).</t>
+        </is>
+      </c>
+      <c r="I5" s="48" t="inlineStr">
+        <is>
+          <t>Clave; 1 a 1 con message_id en el 100 % (misma numeración: C00001 con M00001). Cada hijo tiene la misma cascade_id que su padre en el 100 %.</t>
+        </is>
+      </c>
+      <c r="J5" s="48" t="inlineStr">
+        <is>
+          <t>Agrupa a message_id, hashtag_cluster_ref, topic_code y content_half_life_min, que tienen un solo valor por cascada.</t>
+        </is>
+      </c>
+      <c r="K5" s="48" t="inlineStr">
+        <is>
+          <t>Unidad de validación: el simulador tiene que reproducir la distribución de tamaños (mediana 2, p90 29, p99 188, 40 % de un evento).</t>
+        </is>
+      </c>
+      <c r="L5" s="48" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="M5" s="49" t="inlineStr">
+        <is>
+          <t>C00001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>message_id</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>la publicación: pieza de contenido original, una por cascada</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>clave; 1 a 1 con cascade_id</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>identifica a la entidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="35" t="inlineStr">
+      <c r="B6" s="48" t="inlineStr">
+        <is>
+          <t>La publicación: la pieza de contenido original de la que sale la cascada. Es la entidad del modelo, y «publicar» es el evento que la crea.</t>
+        </is>
+      </c>
+      <c r="C6" s="48" t="inlineStr">
+        <is>
+          <t>texto (identificador)</t>
+        </is>
+      </c>
+      <c r="D6" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="49" t="inlineStr">
+        <is>
+          <t>5.000 valores distintos, uno por cascada</t>
+        </is>
+      </c>
+      <c r="F6" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado.</t>
+        </is>
+      </c>
+      <c r="I6" s="48" t="inlineStr">
+        <is>
+          <t>Clave; 1 a 1 con cascade_id en el 100 %.</t>
+        </is>
+      </c>
+      <c r="J6" s="48" t="inlineStr">
+        <is>
+          <t>Mismo número que cascade_id; toda la cascada comparte el message_id de su semilla.</t>
+        </is>
+      </c>
+      <c r="K6" s="48" t="inlineStr">
+        <is>
+          <t>Identifica a la entidad: cada publicación simulada es un message_id, con el frente de reenvíos vivos como atributo.</t>
+        </is>
+      </c>
+      <c r="L6" s="48" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="M6" s="49" t="inlineStr">
+        <is>
+          <t>M00001</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="71.5" customHeight="1">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>seed_flag</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>marca la publicación original</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>el evento publicar y su tasa horaria</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="B7" s="48" t="inlineStr">
+        <is>
+          <t>Marca el evento que publica la pieza original, la semilla de la cascada: vale 1 ahí y 0 en los reenvíos.</t>
+        </is>
+      </c>
+      <c r="C7" s="48" t="inlineStr">
+        <is>
+          <t>binaria (0/1)</t>
+        </is>
+      </c>
+      <c r="D7" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="49" t="inlineStr">
+        <is>
+          <t>1: 5.000 (7,6 %) · 0: 61.021 (92,4 %)</t>
+        </is>
+      </c>
+      <c r="F7" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado.</t>
+        </is>
+      </c>
+      <c r="I7" s="48" t="inlineStr">
+        <is>
+          <t>Hay exactamente una semilla por cascada. seed_flag = 1 coincide en el 100 % con parent_event_id vacío y con cascade_depth = 0, y en la semilla inter_event_time_min vale siempre 0.</t>
+        </is>
+      </c>
+      <c r="J7" s="48" t="inlineStr">
+        <is>
+          <t>Define dónde empieza el árbol: parent_event_id, cascade_depth e inter_event_time_min se leen distinto en la semilla.</t>
+        </is>
+      </c>
+      <c r="K7" s="48" t="inlineStr">
+        <is>
+          <t>El evento publicar: las fechas de las semillas dan la tasa por hora del día y día de la semana (hoja Llegadas), y su tipo de cuenta, la mezcla de la semilla.</t>
+        </is>
+      </c>
+      <c r="L7" s="48" t="inlineStr">
+        <is>
+          <t>D15 · D17</t>
+        </is>
+      </c>
+      <c r="M7" s="49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>forward_datetime</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>fecha y hora del evento</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>tasa de llegadas; 39 fechas en 2099</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="35" t="inlineStr">
+      <c r="B8" s="48" t="inlineStr">
+        <is>
+          <t>Fecha y hora del evento, con microsegundos: cuándo se publicó la pieza o cuándo se hizo el reenvío.</t>
+        </is>
+      </c>
+      <c r="C8" s="48" t="inlineStr">
+        <is>
+          <t>fecha y hora (texto en el CSV)</t>
+        </is>
+      </c>
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="E8" s="49" t="inlineStr">
+        <is>
+          <t>del 01/03/2025 00:12 al 28/08/2025 10:42 sin las fechas de 2099: 180 días. Semillas por hora: 1,16 de promedio</t>
+        </is>
+      </c>
+      <c r="F8" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="48" t="inlineStr">
+        <is>
+          <t>39 fechas en el año 2099 (2 de ellas en semillas). Se sacan: se toman como faltantes. Además, en 22 hijos la fecha queda antes que la del padre al restar.</t>
+        </is>
+      </c>
+      <c r="I8" s="48" t="inlineStr">
+        <is>
+          <t>La resta con la fecha del padre coincide con inter_event_time_min en el 99,8 % (tolerancia de 0,1 min).</t>
+        </is>
+      </c>
+      <c r="J8" s="48" t="inlineStr">
+        <is>
+          <t>inter_event_time_min es la diferencia con la fecha del padre. En la semilla, la fecha es la del evento publicar.</t>
+        </is>
+      </c>
+      <c r="K8" s="48" t="inlineStr">
+        <is>
+          <t>Tasa de llegadas de publicar por hora del día y día de la semana (valle a las 3 h con 0,51 por hora, pico a las 17 h con 1,62).</t>
+        </is>
+      </c>
+      <c r="L8" s="48" t="inlineStr">
+        <is>
+          <t>D15 · D19</t>
+        </is>
+      </c>
+      <c r="M8" s="49" t="inlineStr">
+        <is>
+          <t>2025-07-15 10:50:54.611892</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>actor_id</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>cuenta que publica o reenvía</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>4.000 cuentas; no es entidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="35" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
+        <is>
+          <t>La cuenta que publica o reenvía en ese evento.</t>
+        </is>
+      </c>
+      <c r="C9" s="48" t="inlineStr">
+        <is>
+          <t>texto (identificador)</t>
+        </is>
+      </c>
+      <c r="D9" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="49" t="inlineStr">
+        <is>
+          <t>4.000 cuentas. Eventos por cuenta: mín 3 · p10 10 · mediana 14 · media 16,5 · p90 21 · máx 77</t>
+        </is>
+      </c>
+      <c r="F9" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado en el identificador. Los seguidores de una misma cuenta cambian entre filas (ver actor_follower_count).</t>
+        </is>
+      </c>
+      <c r="I9" s="48" t="inlineStr">
+        <is>
+          <t>Los atributos fijos de la cuenta (tipo, verificada, antigüedad, seguidos, huella de dispositivo) no cambian entre filas del mismo actor_id en el 100 %.</t>
+        </is>
+      </c>
+      <c r="J9" s="48" t="inlineStr">
+        <is>
+          <t>Agrupa a account_type_code, verified_flag, account_age_days, actor_following_count y device_fingerprint_code, que son de la cuenta.</t>
+        </is>
+      </c>
+      <c r="K9" s="48" t="inlineStr">
+        <is>
+          <t>4.000 cuentas; no es entidad: el enunciado no deja modelar una entidad por usuario. La cuenta entra como atributo del frente, con su tipo y sus seguidores.</t>
+        </is>
+      </c>
+      <c r="L9" s="48" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="M9" s="49" t="inlineStr">
+        <is>
+          <t>U003409</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="98.5" customHeight="1">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>actor_follower_count</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>seguidores</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>impresiones = 0,15 × seguidores</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="35" t="inlineStr">
+      <c r="B10" s="48" t="inlineStr">
+        <is>
+          <t>Cantidad de seguidores de la cuenta que actúa en el evento. Es la audiencia a la que le llega el reenvío.</t>
+        </is>
+      </c>
+      <c r="C10" s="48" t="inlineStr">
+        <is>
+          <t>entero</t>
+        </is>
+      </c>
+      <c r="D10" s="48" t="inlineStr">
+        <is>
+          <t>cuentas</t>
+        </is>
+      </c>
+      <c r="E10" s="49" t="inlineStr">
+        <is>
+          <t>mín 0 · p10 319 · mediana 438 · media 29.264 · p90 45.927 · máx 3.503.446. Por tipo, mediana: BROADCASTER 422.172 · CREATOR 101.192 · resto unos 410</t>
+        </is>
+      </c>
+      <c r="F10" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="48" t="inlineStr">
+        <is>
+          <t>52 eventos con 0 seguidores (52 cuentas distintas, una vez cada una). 3.627 de las 4.000 cuentas tienen más de un valor. Se toma el valor de cada fila como los seguidores al momento del evento; ninguno de los dos casos cambia las estimaciones.</t>
+        </is>
+      </c>
+      <c r="I10" s="48" t="inlineStr">
+        <is>
+          <t>Dato. Que 3.627 cuentas tengan varios valores se explica si es el conteo al momento del evento; es la lectura que usamos.</t>
+        </is>
+      </c>
+      <c r="J10" s="48" t="inlineStr">
+        <is>
+          <t>Impresiones / seguidores: mediana 0,152, entre 0,151 y 0,156 en los cinco tipos. Verificadas: 2 % debajo de 1.000 seguidores y 95 % arriba del millón. Los niveles nano, micro, macro y mega no vienen en los datos: con cortes de 1.000, 10.000, 100.000 y un millón, el 80 % de los eventos queda debajo de todos.</t>
+        </is>
+      </c>
+      <c r="K10" s="48" t="inlineStr">
+        <is>
+          <t>Impresiones = 0,15 × seguidores. Los seguidores se sortean de la empírica por tipo de cuenta.</t>
+        </is>
+      </c>
+      <c r="L10" s="48" t="inlineStr">
+        <is>
+          <t>D12 · D17</t>
+        </is>
+      </c>
+      <c r="M10" s="49" t="inlineStr">
+        <is>
+          <t>208000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="31" customHeight="1">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>actor_following_count</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>a cuántos sigue</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>sin uso</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="35" t="inlineStr">
+      <c r="B11" s="48" t="inlineStr">
+        <is>
+          <t>Cantidad de cuentas a las que sigue la cuenta que actúa.</t>
+        </is>
+      </c>
+      <c r="C11" s="48" t="inlineStr">
+        <is>
+          <t>entero</t>
+        </is>
+      </c>
+      <c r="D11" s="48" t="inlineStr">
+        <is>
+          <t>cuentas</t>
+        </is>
+      </c>
+      <c r="E11" s="49" t="inlineStr">
+        <is>
+          <t>mín 20 · p10 20 · mediana 33 · media 135 · p90 374 · máx 5.325</t>
+        </is>
+      </c>
+      <c r="F11" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado.</t>
+        </is>
+      </c>
+      <c r="I11" s="48" t="inlineStr">
+        <is>
+          <t>Dato. El valor no cambia entre filas de la misma cuenta.</t>
+        </is>
+      </c>
+      <c r="J11" s="48" t="inlineStr">
+        <is>
+          <t>Atributo de la cuenta, como actor_id.</t>
+        </is>
+      </c>
+      <c r="K11" s="48" t="inlineStr">
+        <is>
+          <t>Sin uso: no entra al modelo.</t>
+        </is>
+      </c>
+      <c r="L11" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M11" s="49" t="inlineStr">
+        <is>
+          <t>638</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="112" customHeight="1">
+      <c r="A12" s="47" t="inlineStr">
         <is>
           <t>account_age_days</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>antigüedad de la cuenta</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>señal de coordinación; 514 anteriores a la plataforma</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="35" t="inlineStr">
+      <c r="B12" s="48" t="inlineStr">
+        <is>
+          <t>Antigüedad de la cuenta que actúa, en días.</t>
+        </is>
+      </c>
+      <c r="C12" s="48" t="inlineStr">
+        <is>
+          <t>entero</t>
+        </is>
+      </c>
+      <c r="D12" s="48" t="inlineStr">
+        <is>
+          <t>días</t>
+        </is>
+      </c>
+      <c r="E12" s="49" t="inlineStr">
+        <is>
+          <t>mín 1 · p10 36 · mediana 526 · media 779 · p90 1.834 · máx 6.000. Cuentas de menos de 30 días: 8,2 % de los eventos</t>
+        </is>
+      </c>
+      <c r="F12" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="48" t="inlineStr">
+        <is>
+          <t>514 eventos, de 36 cuentas, tienen más días que los que van de 2013 (cuando arranca la plataforma) a la fecha del evento: cuentas más viejas que la plataforma, hasta 6.000 días. No se corrigen porque no cambian ninguna estimación. El valor no cambia entre eventos de la misma cuenta a lo largo de los 180 días, así que no sabemos a qué fecha está tomado.</t>
+        </is>
+      </c>
+      <c r="I12" s="48" t="inlineStr">
+        <is>
+          <t>Dato.</t>
+        </is>
+      </c>
+      <c r="J12" s="48" t="inlineStr">
+        <is>
+          <t>Cuenta nueva (menos de 30 días): 12,9 % de los eventos en cascadas C2 contra 5,8 % en el resto.</t>
+        </is>
+      </c>
+      <c r="K12" s="48" t="inlineStr">
+        <is>
+          <t>Señal de coordinación. La regla de detección es: al menos una cuenta de menos de 30 días en las primeras 2 h de la publicación (precisión 0,21 y recall 0,47 contra C2).</t>
+        </is>
+      </c>
+      <c r="L12" s="48" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="M12" s="49" t="inlineStr">
+        <is>
+          <t>1253</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="47" t="inlineStr">
         <is>
           <t>verified_flag</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>cuenta verificada</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>probabilidad de remoción (D10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="35" t="inlineStr">
+      <c r="B13" s="48" t="inlineStr">
+        <is>
+          <t>Vale 1 si la cuenta que actúa está verificada.</t>
+        </is>
+      </c>
+      <c r="C13" s="48" t="inlineStr">
+        <is>
+          <t>binaria (0/1)</t>
+        </is>
+      </c>
+      <c r="D13" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="49" t="inlineStr">
+        <is>
+          <t>1: 12,7 % · 0: 87,3 %</t>
+        </is>
+      </c>
+      <c r="F13" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado.</t>
+        </is>
+      </c>
+      <c r="I13" s="48" t="inlineStr">
+        <is>
+          <t>Dato. El valor no cambia entre filas de la misma cuenta.</t>
+        </is>
+      </c>
+      <c r="J13" s="48" t="inlineStr">
+        <is>
+          <t>Va con la audiencia: 2,4 % verificadas debajo de 1.000 seguidores y 94,9 % arriba del millón. No cambia la marca: se marca el 22,9 % de las verificadas y el 23,5 % del resto.</t>
+        </is>
+      </c>
+      <c r="K13" s="48" t="inlineStr">
+        <is>
+          <t>Probabilidad de remoción: a la mitad si la cuenta está verificada. La indulgencia que dice el enunciado no se ve en la marca, así que va en la remoción.</t>
+        </is>
+      </c>
+      <c r="L13" s="48" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="M13" s="49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="98.5" customHeight="1">
+      <c r="A14" s="47" t="inlineStr">
         <is>
           <t>account_type_code</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>BROADCASTER · CREATOR · AGGREGATOR · LURKER · STANDARD</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>por los roles del enunciado</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>el factor que más mueve R</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="35" t="inlineStr">
+      <c r="B14" s="48" t="inlineStr">
+        <is>
+          <t>Rol de la cuenta: BROADCASTER es el difusor masivo, CREATOR el creador, AGGREGATOR el reposteador, LURKER el durmiente y STANDARD la cuenta estándar.</t>
+        </is>
+      </c>
+      <c r="C14" s="48" t="inlineStr">
+        <is>
+          <t>categórica (5 valores)</t>
+        </is>
+      </c>
+      <c r="D14" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="49" t="inlineStr">
+        <is>
+          <t>En todos los eventos: STANDARD 49,1 % · AGGREGATOR 22,0 % · LURKER 19,2 % · CREATOR 6,1 % · BROADCASTER 3,6 %. En semillas: STANDARD 39 % · AGGREGATOR 18 % · CREATOR 17 % · LURKER 15 % · BROADCASTER 12 %. En reenvíos: STANDARD 50 % · AGGREGATOR 22 % · LURKER 20 % · CREATOR 5 % · BROADCASTER 3 %</t>
+        </is>
+      </c>
+      <c r="F14" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado: siempre en mayúsculas y sin faltantes.</t>
+        </is>
+      </c>
+      <c r="I14" s="48" t="inlineStr">
+        <is>
+          <t>Por los roles que nombra el enunciado (§5); el mapeo de cada código a un rol es nuestro. El valor no cambia entre filas de la misma cuenta.</t>
+        </is>
+      </c>
+      <c r="J14" s="48" t="inlineStr">
+        <is>
+          <t>Hijos medios por tipo, sin las 14 cascadas cortadas: BROADCASTER 4,44 · CREATOR 3,53 · AGGREGATOR 0,58 · LURKER 0,59 · STANDARD 0,59. Los roles no coinciden con los niveles de audiencia: son dos variables distintas.</t>
+        </is>
+      </c>
+      <c r="K14" s="48" t="inlineStr">
+        <is>
+          <t>El factor que más mueve R. Tipo de la semilla (discreta) y tipos del frente hijo (multinomial fija), con R por tipo.</t>
+        </is>
+      </c>
+      <c r="L14" s="48" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="M14" s="49" t="inlineStr">
+        <is>
+          <t>BROADCASTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44.5" customHeight="1">
+      <c r="A15" s="47" t="inlineStr">
         <is>
           <t>parent_event_id</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>evento padre</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>estructura</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>reconstruye el árbol y define R</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="35" t="inlineStr">
+      <c r="B15" s="48" t="inlineStr">
+        <is>
+          <t>El event_id del evento del que sale este reenvío: quién le pasó la pieza a esta cuenta.</t>
+        </is>
+      </c>
+      <c r="C15" s="48" t="inlineStr">
+        <is>
+          <t>texto (identificador)</t>
+        </is>
+      </c>
+      <c r="D15" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="49" t="inlineStr">
+        <is>
+          <t>25.186 padres distintos (los eventos que tuvieron al menos un hijo)</t>
+        </is>
+      </c>
+      <c r="F15" s="50" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G15" s="51" t="n">
+        <v>0.07573347874161251</v>
+      </c>
+      <c r="H15" s="48" t="inlineStr">
+        <is>
+          <t>Vacío en las 5.000 semillas, que no tienen padre: no es un faltante.</t>
+        </is>
+      </c>
+      <c r="I15" s="48" t="inlineStr">
+        <is>
+          <t>No hay padres fuera de la muestra. El padre está siempre en la misma cascada (100 %).</t>
+        </is>
+      </c>
+      <c r="J15" s="48" t="inlineStr">
+        <is>
+          <t>Contar cuántas veces aparece un event_id como padre da reshare_count_from_actor en el 100 %. cascade_depth es la del padre + 1.</t>
+        </is>
+      </c>
+      <c r="K15" s="48" t="inlineStr">
+        <is>
+          <t>Reconstruye el árbol y define R, los hijos por evento.</t>
+        </is>
+      </c>
+      <c r="L15" s="48" t="inlineStr">
+        <is>
+          <t>D16</t>
+        </is>
+      </c>
+      <c r="M15" s="49" t="inlineStr">
+        <is>
+          <t>E0000002</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="71.5" customHeight="1">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>cascade_depth</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>generación</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>es la del padre + 1 en el 100 %</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>decaimiento (D18)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="35" t="inlineStr">
+      <c r="B16" s="48" t="inlineStr">
+        <is>
+          <t>Generación del evento dentro de la cascada: 0 es la semilla, 1 los reenvíos directos, 2 los reenvíos de reenvíos, y así.</t>
+        </is>
+      </c>
+      <c r="C16" s="48" t="inlineStr">
+        <is>
+          <t>entero</t>
+        </is>
+      </c>
+      <c r="D16" s="48" t="inlineStr">
+        <is>
+          <t>generaciones</t>
+        </is>
+      </c>
+      <c r="E16" s="49" t="inlineStr">
+        <is>
+          <t>de 0 a 15. Eventos por generación: 0: 5.000 · 1: 11.961 · 2: 12.483 · 3: 11.300 · 4: 9.605 · 5: 6.481 · 6: 4.328 · 7: 2.457 · 8: 1.365 · 9: 637 · 10: 253 · 11: 98 · 12: 36 · 13: 11 · 14: 3 · 15: 3</t>
+        </is>
+      </c>
+      <c r="F16" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado.</t>
+        </is>
+      </c>
+      <c r="I16" s="48" t="inlineStr">
+        <is>
+          <t>Es la del padre + 1 en el 100 % de los reenvíos.</t>
+        </is>
+      </c>
+      <c r="J16" s="48" t="inlineStr">
+        <is>
+          <t>Hijos medios por generación, sin las cortadas: 2,35 · 1,00 · 0,85 · 0,78 · 0,68 · … · 0,37 en la 11. De la 12 en adelante hay menos de 40 eventos.</t>
+        </is>
+      </c>
+      <c r="K16" s="48" t="inlineStr">
+        <is>
+          <t>Decaimiento por generación δ(g): hijos medios de g sobre los de g = 1.</t>
+        </is>
+      </c>
+      <c r="L16" s="48" t="inlineStr">
+        <is>
+          <t>D18</t>
+        </is>
+      </c>
+      <c r="M16" s="49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="47" t="inlineStr">
         <is>
           <t>reshare_count_from_actor</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>hijos del evento</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>coincide 100 % con contar parent_event_id</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>chequeo</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="35" t="inlineStr">
+      <c r="B17" s="48" t="inlineStr">
+        <is>
+          <t>Cantidad de reenvíos directos que tuvo el evento: sus hijos en el árbol.</t>
+        </is>
+      </c>
+      <c r="C17" s="48" t="inlineStr">
+        <is>
+          <t>entero</t>
+        </is>
+      </c>
+      <c r="D17" s="48" t="inlineStr">
+        <is>
+          <t>reenvíos</t>
+        </is>
+      </c>
+      <c r="E17" s="49" t="inlineStr">
+        <is>
+          <t>mín 0 · p10 0 · mediana 0 · media 0,92 · p90 2 · máx 45. Media sin las cortadas: 0,916</t>
+        </is>
+      </c>
+      <c r="F17" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado.</t>
+        </is>
+      </c>
+      <c r="I17" s="48" t="inlineStr">
+        <is>
+          <t>Coincide en el 100 % con contar cuántas veces aparece el event_id como parent_event_id: es redundante.</t>
+        </is>
+      </c>
+      <c r="J17" s="48" t="inlineStr">
+        <is>
+          <t>Es la cuenta de hijos de parent_event_id. Varianza sobre media, sin las cortadas: 4,8; con todas: 5,1. La media 0,92 da un proceso subcrítico: coincide con 1 − 1/tamaño medio.</t>
+        </is>
+      </c>
+      <c r="K17" s="48" t="inlineStr">
+        <is>
+          <t>Chequeo. R y su dispersión salen de acá o de parent_event_id, que es lo mismo.</t>
+        </is>
+      </c>
+      <c r="L17" s="48" t="inlineStr">
+        <is>
+          <t>D16</t>
+        </is>
+      </c>
+      <c r="M17" s="49" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="47" t="inlineStr">
         <is>
           <t>impressions</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>impresiones del evento</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>VR y economía; 625 faltantes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="35" t="inlineStr">
+      <c r="B18" s="48" t="inlineStr">
+        <is>
+          <t>Veces que se mostró el evento: cuánta gente vio ese reenvío.</t>
+        </is>
+      </c>
+      <c r="C18" s="48" t="inlineStr">
+        <is>
+          <t>decimal (en la práctica, entero)</t>
+        </is>
+      </c>
+      <c r="D18" s="48" t="inlineStr">
+        <is>
+          <t>impresiones</t>
+        </is>
+      </c>
+      <c r="E18" s="49" t="inlineStr">
+        <is>
+          <t>mín 1 · p10 18 · mediana 81 · media 5.454 · p90 5.446 · máx 2.323.023</t>
+        </is>
+      </c>
+      <c r="F18" s="50" t="n">
+        <v>625</v>
+      </c>
+      <c r="G18" s="51" t="n">
+        <v>0.009466684842701564</v>
+      </c>
+      <c r="H18" s="48" t="inlineStr">
+        <is>
+          <t>625 faltantes: se dejan como faltantes, no se imputan. 51 eventos tienen más impresiones que seguidores; no se tocan.</t>
+        </is>
+      </c>
+      <c r="I18" s="48" t="inlineStr">
+        <is>
+          <t>Dato. Impresiones / seguidores: mediana 0,15, p10 0,04, p90 0,38.</t>
+        </is>
+      </c>
+      <c r="J18" s="48" t="inlineStr">
+        <is>
+          <t>Proporcional a actor_follower_count (0,15, parejo en los cinco tipos). Una regresión por el origen da 0,19, pero la arrastran las cuentas grandes, así que usamos la mediana.</t>
+        </is>
+      </c>
+      <c r="K18" s="48" t="inlineStr">
+        <is>
+          <t>VR y economía: impresiones nocivas servidas e impresiones legítimas perdidas. La degradación baja el factor 0,15.</t>
+        </is>
+      </c>
+      <c r="L18" s="48" t="inlineStr">
+        <is>
+          <t>D4 · D12</t>
+        </is>
+      </c>
+      <c r="M18" s="49" t="inlineStr">
+        <is>
+          <t>139470</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44.5" customHeight="1">
+      <c r="A19" s="47" t="inlineStr">
         <is>
           <t>likes</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="48" t="inlineStr">
+        <is>
+          <t>Cantidad de «me gusta» que recibió el evento.</t>
+        </is>
+      </c>
+      <c r="C19" s="48" t="inlineStr">
+        <is>
+          <t>entero</t>
+        </is>
+      </c>
+      <c r="D19" s="48" t="inlineStr">
         <is>
           <t>me gusta</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>sin uso</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="35" t="inlineStr">
+      <c r="E19" s="49" t="inlineStr">
+        <is>
+          <t>mín 0 · p10 0 · mediana 1 · media 65 · p90 45 · máx 38.029</t>
+        </is>
+      </c>
+      <c r="F19" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="48" t="inlineStr">
+        <is>
+          <t>Sin faltantes. 49 eventos tienen más me gusta que impresiones; no se tocan porque la columna no se usa.</t>
+        </is>
+      </c>
+      <c r="I19" s="48" t="inlineStr">
+        <is>
+          <t>Dato.</t>
+        </is>
+      </c>
+      <c r="J19" s="48" t="inlineStr">
+        <is>
+          <t>Me gusta / impresiones: mediana 0,76 %.</t>
+        </is>
+      </c>
+      <c r="K19" s="48" t="inlineStr">
+        <is>
+          <t>Sin uso: no entra al modelo.</t>
+        </is>
+      </c>
+      <c r="L19" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M19" s="49" t="inlineStr">
+        <is>
+          <t>3156</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44.5" customHeight="1">
+      <c r="A20" s="47" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="48" t="inlineStr">
+        <is>
+          <t>Cantidad de comentarios que recibió el evento.</t>
+        </is>
+      </c>
+      <c r="C20" s="48" t="inlineStr">
+        <is>
+          <t>decimal (en la práctica, entero)</t>
+        </is>
+      </c>
+      <c r="D20" s="48" t="inlineStr">
         <is>
           <t>comentarios</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>sin uso; 937 faltantes</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="35" t="inlineStr">
+      <c r="E20" s="49" t="inlineStr">
+        <is>
+          <t>mín 0 · p10 0 · mediana 0 · media 12 · p90 7 · máx 8.223</t>
+        </is>
+      </c>
+      <c r="F20" s="50" t="n">
+        <v>936</v>
+      </c>
+      <c r="G20" s="51" t="n">
+        <v>0.01417730722042986</v>
+      </c>
+      <c r="H20" s="48" t="inlineStr">
+        <is>
+          <t>936 faltantes. No se imputan porque la columna no se usa.</t>
+        </is>
+      </c>
+      <c r="I20" s="48" t="inlineStr">
+        <is>
+          <t>Dato.</t>
+        </is>
+      </c>
+      <c r="J20" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K20" s="48" t="inlineStr">
+        <is>
+          <t>Sin uso: no entra al modelo.</t>
+        </is>
+      </c>
+      <c r="L20" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M20" s="49" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44.5" customHeight="1">
+      <c r="A21" s="47" t="inlineStr">
         <is>
           <t>dwell_time_sec</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>tiempo de visualización</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>sin uso; 2.008 faltantes y 66 negativos</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="35" t="inlineStr">
+      <c r="B21" s="48" t="inlineStr">
+        <is>
+          <t>Tiempo que la gente se quedó mirando la pieza en ese evento, en segundos.</t>
+        </is>
+      </c>
+      <c r="C21" s="48" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="D21" s="48" t="inlineStr">
+        <is>
+          <t>segundos</t>
+        </is>
+      </c>
+      <c r="E21" s="49" t="inlineStr">
+        <is>
+          <t>mín 1,0 · p10 13,4 · mediana 55,0 · media 100,2 · p90 227,0 · máx 6.140,1. Sin los negativos</t>
+        </is>
+      </c>
+      <c r="F21" s="50" t="n">
+        <v>2005</v>
+      </c>
+      <c r="G21" s="51" t="n">
+        <v>0.03036912497538662</v>
+      </c>
+      <c r="H21" s="48" t="inlineStr">
+        <is>
+          <t>2.005 faltantes y 66 negativos (entre −49,8 y −2,4 s), que se dejan fuera. Es la columna con más faltantes.</t>
+        </is>
+      </c>
+      <c r="I21" s="48" t="inlineStr">
+        <is>
+          <t>Dato.</t>
+        </is>
+      </c>
+      <c r="J21" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K21" s="48" t="inlineStr">
+        <is>
+          <t>Sin uso: no entra al modelo.</t>
+        </is>
+      </c>
+      <c r="L21" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M21" s="49" t="inlineStr">
+        <is>
+          <t>24,8</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="47" t="inlineStr">
         <is>
           <t>inter_event_time_min</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>minutos desde el padre</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>coincide 99,8 % con la resta de fechas</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>tiempo entre generaciones (D19)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="35" t="inlineStr">
+      <c r="B22" s="48" t="inlineStr">
+        <is>
+          <t>Minutos entre el evento padre y este reenvío: cuánto tardó la pieza en saltar una generación. En la semilla vale 0.</t>
+        </is>
+      </c>
+      <c r="C22" s="48" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="D22" s="48" t="inlineStr">
+        <is>
+          <t>minutos</t>
+        </is>
+      </c>
+      <c r="E22" s="49" t="inlineStr">
+        <is>
+          <t>En reenvíos: mín −9,3 · p10 1,2 · mediana 42,7 · media 69,7 · p90 150,3 · máx 57.241,9</t>
+        </is>
+      </c>
+      <c r="F22" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="48" t="inlineStr">
+        <is>
+          <t>39 valores negativos (entre −9,3 y −1,0 min), que se dejan fuera. Aparte, en 22 hijos la resta de fechas da negativa aunque la columna no; no se superponen con los 39.</t>
+        </is>
+      </c>
+      <c r="I22" s="48" t="inlineStr">
+        <is>
+          <t>Coincide en el 99,8 % con restar forward_datetime del padre (tolerancia de 0,1 min). De los 98 que no coinciden, 59 tienen una fecha de 2099 en el hijo o en el padre.</t>
+        </is>
+      </c>
+      <c r="J22" s="48" t="inlineStr">
+        <is>
+          <t>Diferencia de forward_datetime entre hijo y padre. Vale 0 en todas las semillas (seed_flag = 1).</t>
+        </is>
+      </c>
+      <c r="K22" s="48" t="inlineStr">
+        <is>
+          <t>Tiempo entre generaciones: gamma de forma 0,55 y escala 128 min (media 70, mediana 43). No puede ser Erlang (hoja Ajuste D19).</t>
+        </is>
+      </c>
+      <c r="L22" s="48" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
+      <c r="M22" s="49" t="inlineStr">
+        <is>
+          <t>15,41</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="47" t="inlineStr">
         <is>
           <t>content_half_life_min</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>vida media de la pieza</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>dato, uno por cascada</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>no correlaciona con el tamaño (D18)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="35" t="inlineStr">
+      <c r="B23" s="48" t="inlineStr">
+        <is>
+          <t>Vida media de la pieza, en minutos. Es un atributo de la publicación, no del reenvío: hay un solo valor por cascada.</t>
+        </is>
+      </c>
+      <c r="C23" s="48" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="D23" s="48" t="inlineStr">
+        <is>
+          <t>minutos</t>
+        </is>
+      </c>
+      <c r="E23" s="49" t="inlineStr">
+        <is>
+          <t>Por cascada: mín 15,0 · p10 72,7 · mediana 219,4 · media 328,9 · p90 691,0 · máx 4.993,5</t>
+        </is>
+      </c>
+      <c r="F23" s="50" t="n">
+        <v>666</v>
+      </c>
+      <c r="G23" s="51" t="n">
+        <v>0.01008769936838279</v>
+      </c>
+      <c r="H23" s="48" t="inlineStr">
+        <is>
+          <t>666 filas sin valor, repartidas en 466 cascadas. En 448 de ellas otras filas de la misma cascada sí lo tienen; sólo 18 cascadas no lo tienen en ninguna fila.</t>
+        </is>
+      </c>
+      <c r="I23" s="48" t="inlineStr">
+        <is>
+          <t>Dato. Un solo valor por cascada: ninguna tiene dos valores distintos.</t>
+        </is>
+      </c>
+      <c r="J23" s="48" t="inlineStr">
+        <is>
+          <t>No correlaciona con el tamaño de la cascada: Spearman 0,04. Los hijos por generación sí caen (cascade_depth).</t>
+        </is>
+      </c>
+      <c r="K23" s="48" t="inlineStr">
+        <is>
+          <t>No correlaciona con el tamaño, así que el decaimiento va por generación y la vida media entra sólo en sensibilidad.</t>
+        </is>
+      </c>
+      <c r="L23" s="48" t="inlineStr">
+        <is>
+          <t>D18</t>
+        </is>
+      </c>
+      <c r="M23" s="49" t="inlineStr">
+        <is>
+          <t>250,1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="47" t="inlineStr">
         <is>
           <t>content_type_code</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>formato</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>multiplicador chico de R: 0,77 a 0,96</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="35" t="inlineStr">
+      <c r="B24" s="48" t="inlineStr">
+        <is>
+          <t>Formato de la pieza. Por el nombre de los códigos: imagen con texto (meme), video corto, texto, captura de pantalla, link externo y encuesta.</t>
+        </is>
+      </c>
+      <c r="C24" s="48" t="inlineStr">
+        <is>
+          <t>categórica (6 valores)</t>
+        </is>
+      </c>
+      <c r="D24" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="49" t="inlineStr">
+        <is>
+          <t>Normalizado a mayúsculas: IMG-MACRO 39,3 % · VID-SHORT 34,6 % · TXT 9,9 % · SCREENSHOT 8,3 % · LINK-EXT 4,6 % · POLL 3,3 %</t>
+        </is>
+      </c>
+      <c r="F24" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="48" t="inlineStr">
+        <is>
+          <t>4.644 celdas en minúscula (img-macro, vid-short…). Se pasan a mayúsculas; con eso queda un solo formato por cascada.</t>
+        </is>
+      </c>
+      <c r="I24" s="48" t="inlineStr">
+        <is>
+          <t>Dato. Normalizado, tiene un solo valor por cascada.</t>
+        </is>
+      </c>
+      <c r="J24" s="48" t="inlineStr">
+        <is>
+          <t>Hijos medios por formato, sin las cortadas: LINK-EXT 0,77 · TXT 0,83 · POLL 0,88 · SCREENSHOT 0,89 · IMG-MACRO 0,94 · VID-SHORT 0,95.</t>
+        </is>
+      </c>
+      <c r="K24" s="48" t="inlineStr">
+        <is>
+          <t>Multiplicador chico de R: 0,77 a 0,95.</t>
+        </is>
+      </c>
+      <c r="L24" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M24" s="49" t="inlineStr">
+        <is>
+          <t>IMG-MACRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="112" customHeight="1">
+      <c r="A25" s="47" t="inlineStr">
         <is>
           <t>topic_code</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>tema: DISARM-* u ORG-*</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>marco de DISARM</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>candidato a «nocivo» (D8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="35" t="inlineStr">
+      <c r="B25" s="48" t="inlineStr">
+        <is>
+          <t>Tema de la pieza. Los DISARM-* son técnicas de desinformación del marco de DISARM Foundation: T0003 Leverage Existing Narratives, T0023 Distort Facts, T0039 Bait Influencer, T0049 Flood Information Space y T0049.003 Bots Amplify via Automated Forwarding and Reposting. Los ORG-* son temas orgánicos: POL, HLTH, FIN, CELEB y LOCAL.</t>
+        </is>
+      </c>
+      <c r="C25" s="48" t="inlineStr">
+        <is>
+          <t>categórica (10 valores)</t>
+        </is>
+      </c>
+      <c r="D25" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="49" t="inlineStr">
+        <is>
+          <t>ORG-POL 16,8 % · ORG-HLTH 13,7 % · ORG-FIN 10,7 % · ORG-CELEB 10,3 % · DISARM-T0003 9,3 % · ORG-LOCAL 8,9 % · DISARM-T0023 8,8 % · DISARM-T0049 8,2 % · DISARM-T0039 7,1 % · DISARM-T0049.003 6,3 %. DISARM en total: 40 % de los eventos</t>
+        </is>
+      </c>
+      <c r="F25" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado.</t>
+        </is>
+      </c>
+      <c r="I25" s="48" t="inlineStr">
+        <is>
+          <t>Los DISARM, por el repo oficial de DISARM Foundation (consultado el 15/9). Los ORG, por contraste. Hipótesis: DISARM = nocivo y ORG = legítimo. Un solo valor por cascada.</t>
+        </is>
+      </c>
+      <c r="J25" s="48" t="inlineStr">
+        <is>
+          <t>Marcado por tema: DISARM entre 32 % y 36 %; ORG entre 14 % y 22 %. Con DISARM como nocivo, Centinela da precisión 0,57 y recall 0,34, contra 0,72 y 0,63 del CSV de parámetros.</t>
+        </is>
+      </c>
+      <c r="K25" s="48" t="inlineStr">
+        <is>
+          <t>Candidato a «nocivo». Probabilidad de marca por tema y quintil de toxicidad. Temas sensibles (DISARM, POL, HLTH) para la remoción.</t>
+        </is>
+      </c>
+      <c r="L25" s="48" t="inlineStr">
+        <is>
+          <t>D8 · D10</t>
+        </is>
+      </c>
+      <c r="M25" s="49" t="inlineStr">
+        <is>
+          <t>DISARM-T0023</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44.5" customHeight="1">
+      <c r="A26" s="47" t="inlineStr">
         <is>
           <t>toxicity_index</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>puntaje de Centinela</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>dato, nunca falta</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>probabilidad de marca; el otro candidato a «nocivo»</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="35" t="inlineStr">
+      <c r="B26" s="48" t="inlineStr">
+        <is>
+          <t>Puntaje de nocividad que Centinela le pone a cada evento, entre 0 y 1.</t>
+        </is>
+      </c>
+      <c r="C26" s="48" t="inlineStr">
+        <is>
+          <t>decimal (0 a 1)</t>
+        </is>
+      </c>
+      <c r="D26" s="48" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="E26" s="49" t="inlineStr">
+        <is>
+          <t>mín 0,00 · p10 0,11 · mediana 0,34 · media 0,36 · p90 0,63 · máx 1,00</t>
+        </is>
+      </c>
+      <c r="F26" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="48" t="inlineStr">
+        <is>
+          <t>Sin faltantes y siempre entre 0 y 1: nada detectado.</t>
+        </is>
+      </c>
+      <c r="I26" s="48" t="inlineStr">
+        <is>
+          <t>Dato. Nunca falta, como dice el enunciado de Centinela. Cambia entre eventos de la misma cascada: es del evento, no de la pieza.</t>
+        </is>
+      </c>
+      <c r="J26" s="48" t="inlineStr">
+        <is>
+          <t>Marcado por quintil de toxicidad: 12 % · 18 % · 23 % · 29 % · 36 %. Spearman con sentiment_score: −0,21.</t>
+        </is>
+      </c>
+      <c r="K26" s="48" t="inlineStr">
+        <is>
+          <t>Probabilidad de marca y probabilidad de remoción (toxicidad × 1,5 en temas sensibles o × 1). Es el otro candidato a «nocivo».</t>
+        </is>
+      </c>
+      <c r="L26" s="48" t="inlineStr">
+        <is>
+          <t>D8 · D10</t>
+        </is>
+      </c>
+      <c r="M26" s="49" t="inlineStr">
+        <is>
+          <t>0,66</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="31" customHeight="1">
+      <c r="A27" s="47" t="inlineStr">
         <is>
           <t>sentiment_score</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>sentimiento</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>sin uso; 1.347 faltantes</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="35" t="inlineStr">
+      <c r="B27" s="48" t="inlineStr">
+        <is>
+          <t>Sentimiento del contenido del evento, de −1 (negativo) a 1 (positivo).</t>
+        </is>
+      </c>
+      <c r="C27" s="48" t="inlineStr">
+        <is>
+          <t>decimal (−1 a 1)</t>
+        </is>
+      </c>
+      <c r="D27" s="48" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="E27" s="49" t="inlineStr">
+        <is>
+          <t>mín −1,00 · p10 −0,76 · mediana −0,29 · media −0,29 · p90 0,18 · máx 1,00</t>
+        </is>
+      </c>
+      <c r="F27" s="50" t="n">
+        <v>1344</v>
+      </c>
+      <c r="G27" s="51" t="n">
+        <v>0.02035715908574545</v>
+      </c>
+      <c r="H27" s="48" t="inlineStr">
+        <is>
+          <t>1.344 faltantes. No se imputan porque la columna no se usa.</t>
+        </is>
+      </c>
+      <c r="I27" s="48" t="inlineStr">
+        <is>
+          <t>Dato.</t>
+        </is>
+      </c>
+      <c r="J27" s="48" t="inlineStr">
+        <is>
+          <t>Relación débil y negativa con toxicity_index.</t>
+        </is>
+      </c>
+      <c r="K27" s="48" t="inlineStr">
+        <is>
+          <t>Sin uso: no entra al modelo.</t>
+        </is>
+      </c>
+      <c r="L27" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M27" s="49" t="inlineStr">
+        <is>
+          <t>0,198</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="58" customHeight="1">
+      <c r="A28" s="47" t="inlineStr">
         <is>
           <t>platform_surface_code</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>FEED · GROUP · STORY · DM · REPOST</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>multiplicador de R: 0,55 a 1,13</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="35" t="inlineStr">
+      <c r="B28" s="48" t="inlineStr">
+        <is>
+          <t>Superficie de la plataforma donde ocurre el evento. Por el nombre de los códigos: el feed, un grupo, una historia, un mensaje directo o un repost.</t>
+        </is>
+      </c>
+      <c r="C28" s="48" t="inlineStr">
+        <is>
+          <t>categórica (5 valores)</t>
+        </is>
+      </c>
+      <c r="D28" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="49" t="inlineStr">
+        <is>
+          <t>Normalizado a mayúsculas: FEED 42,0 % · GROUP 17,7 % · STORY 16,4 % · REPOST 13,9 % · DM 10,0 %</t>
+        </is>
+      </c>
+      <c r="F28" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="48" t="inlineStr">
+        <is>
+          <t>4.629 celdas en minúscula. Se pasan a mayúsculas.</t>
+        </is>
+      </c>
+      <c r="I28" s="48" t="inlineStr">
+        <is>
+          <t>Dato. Cambia entre eventos de la misma cascada.</t>
+        </is>
+      </c>
+      <c r="J28" s="48" t="inlineStr">
+        <is>
+          <t>Hijos medios por superficie, sin las cortadas: DM 0,55 · STORY 0,76 · FEED 0,94 · REPOST 1,03 · GROUP 1,12.</t>
+        </is>
+      </c>
+      <c r="K28" s="48" t="inlineStr">
+        <is>
+          <t>Multiplicador de R: 0,55 a 1,12. Pesa menos que el tipo de cuenta.</t>
+        </is>
+      </c>
+      <c r="L28" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M28" s="49" t="inlineStr">
+        <is>
+          <t>FEED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="58" customHeight="1">
+      <c r="A29" s="47" t="inlineStr">
         <is>
           <t>language_code</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>idioma</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>dato sucio (es · ES · es-AR)</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>sin uso</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="35" t="inlineStr">
+      <c r="B29" s="48" t="inlineStr">
+        <is>
+          <t>Idioma del evento.</t>
+        </is>
+      </c>
+      <c r="C29" s="48" t="inlineStr">
+        <is>
+          <t>categórica</t>
+        </is>
+      </c>
+      <c r="D29" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="49" t="inlineStr">
+        <is>
+          <t>Normalizado a minúsculas: es 46,2 % · pt 20,4 % · en 19,2 % · es-ar 9,5 % · fr 4,7 %</t>
+        </is>
+      </c>
+      <c r="F29" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="48" t="inlineStr">
+        <is>
+          <t>4.551 celdas en mayúscula (ES, PT, EN, ES-AR, FR). Se pasan a minúsculas. es y es-ar quedan separados: como la columna no se usa, no hizo falta decidir si son el mismo idioma.</t>
+        </is>
+      </c>
+      <c r="I29" s="48" t="inlineStr">
+        <is>
+          <t>Dato sucio (es · ES · es-AR).</t>
+        </is>
+      </c>
+      <c r="J29" s="48" t="inlineStr">
+        <is>
+          <t>Cambia entre eventos de la misma cascada.</t>
+        </is>
+      </c>
+      <c r="K29" s="48" t="inlineStr">
+        <is>
+          <t>Sin uso: no entra al modelo.</t>
+        </is>
+      </c>
+      <c r="L29" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M29" s="49" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="58" customHeight="1">
+      <c r="A30" s="47" t="inlineStr">
         <is>
           <t>hashtag_cluster_ref</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>identificador de campaña</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>hipótesis: el sufijo C2 es coordinación</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>qué es coordinada (D11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="35" t="inlineStr">
+      <c r="B30" s="48" t="inlineStr">
+        <is>
+          <t>Identificador de campaña, uno por cascada. Tiene la forma HC-número-sufijo (por ejemplo HC-5338-B).</t>
+        </is>
+      </c>
+      <c r="C30" s="48" t="inlineStr">
+        <is>
+          <t>texto (identificador)</t>
+        </is>
+      </c>
+      <c r="D30" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="49" t="inlineStr">
+        <is>
+          <t>4.845 valores distintos. Cascadas por sufijo: A 579 · B 534 · C2 514 · D 594 · E 550 · F 543 · G 578 · H 571 · K 537</t>
+        </is>
+      </c>
+      <c r="F30" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado. Hay un valor por cascada, pero 149 valores aparecen en más de una cascada.</t>
+        </is>
+      </c>
+      <c r="I30" s="48" t="inlineStr">
+        <is>
+          <t>Hipótesis: el sufijo C2 marca coordinación. Es el único sufijo de dos caracteres y tiene las 14 cascadas cortadas en 500.</t>
+        </is>
+      </c>
+      <c r="J30" s="48" t="inlineStr">
+        <is>
+          <t>Cascadas C2: 42,8 eventos de media contra 9,8 del resto, y 13 % de cuentas nuevas contra 6 %.</t>
+        </is>
+      </c>
+      <c r="K30" s="48" t="inlineStr">
+        <is>
+          <t>Qué es coordinada: C2 es la referencia contra la que se mide la regla de detección (C2 + cuenta nueva, con error). También define las 14 cascadas cortadas.</t>
+        </is>
+      </c>
+      <c r="L30" s="48" t="inlineStr">
+        <is>
+          <t>D11 · D14</t>
+        </is>
+      </c>
+      <c r="M30" s="49" t="inlineStr">
+        <is>
+          <t>HC-5338-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="31" customHeight="1">
+      <c r="A31" s="47" t="inlineStr">
         <is>
           <t>device_fingerprint_code</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>rasgo del dispositivo</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>no separa: el 98 % está en más de 3 cascadas</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="35" t="inlineStr">
+      <c r="B31" s="48" t="inlineStr">
+        <is>
+          <t>Rasgo del dispositivo desde el que actúa la cuenta.</t>
+        </is>
+      </c>
+      <c r="C31" s="48" t="inlineStr">
+        <is>
+          <t>texto (identificador)</t>
+        </is>
+      </c>
+      <c r="D31" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="49" t="inlineStr">
+        <is>
+          <t>3.989 valores distintos, casi uno por cuenta (4.000)</t>
+        </is>
+      </c>
+      <c r="F31" s="50" t="n">
+        <v>1324</v>
+      </c>
+      <c r="G31" s="51" t="n">
+        <v>0.02005422517077899</v>
+      </c>
+      <c r="H31" s="48" t="inlineStr">
+        <is>
+          <t>1.324 faltantes. No se imputan porque la columna no se usa.</t>
+        </is>
+      </c>
+      <c r="I31" s="48" t="inlineStr">
+        <is>
+          <t>Dato. Cada cuenta tiene una sola huella; 11 huellas aparecen en más de una cuenta.</t>
+        </is>
+      </c>
+      <c r="J31" s="48" t="inlineStr">
+        <is>
+          <t>El 99,9 % de las huellas aparece en más de tres cascadas, dentro y fuera de C2.</t>
+        </is>
+      </c>
+      <c r="K31" s="48" t="inlineStr">
+        <is>
+          <t>No separa: sola no sirve para detectar coordinación, así que no entra al modelo.</t>
+        </is>
+      </c>
+      <c r="L31" s="48" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="M31" s="49" t="inlineStr">
+        <is>
+          <t>DFP-F6FED</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="58" customHeight="1">
+      <c r="A32" s="47" t="inlineStr">
         <is>
           <t>moderation_flag</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>marcada por Centinela</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>tasa a reproducir</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="35" t="inlineStr">
+      <c r="B32" s="48" t="inlineStr">
+        <is>
+          <t>Vale 1 si Centinela marcó el evento y lo mandó a revisión.</t>
+        </is>
+      </c>
+      <c r="C32" s="48" t="inlineStr">
+        <is>
+          <t>binaria (0/1)</t>
+        </is>
+      </c>
+      <c r="D32" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="49" t="inlineStr">
+        <is>
+          <t>1: 15.445 (23,4 %) · 0: 50.576 (76,6 %)</t>
+        </is>
+      </c>
+      <c r="F32" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="48" t="inlineStr">
+        <is>
+          <t>Nada detectado.</t>
+        </is>
+      </c>
+      <c r="I32" s="48" t="inlineStr">
+        <is>
+          <t>Dato. moderation_latency_min es mayor que 0 sólo en eventos marcados (100 %). Cambia entre eventos de la misma cascada.</t>
+        </is>
+      </c>
+      <c r="J32" s="48" t="inlineStr">
+        <is>
+          <t>Sube con toxicity_index (12 % a 36 % por quintil) y con el tema (DISARM el doble que ORG). El 11 % de los hijos de un evento marcado nace después de la acción: no todo lo marcado se remueve.</t>
+        </is>
+      </c>
+      <c r="K32" s="48" t="inlineStr">
+        <is>
+          <t>Tasa a reproducir: probabilidad de marca por tema y quintil de toxicidad (hoja Marca). Los ítems marcados son los que entran a la cola.</t>
+        </is>
+      </c>
+      <c r="L32" s="48" t="inlineStr">
+        <is>
+          <t>D8 · D10</t>
+        </is>
+      </c>
+      <c r="M32" s="49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="58" customHeight="1">
+      <c r="A33" s="47" t="inlineStr">
         <is>
           <t>moderation_latency_min</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>minutos hasta la acción</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>dato</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>salida, no entrada: objetivo de validación</t>
+      <c r="B33" s="48" t="inlineStr">
+        <is>
+          <t>Minutos desde el evento hasta la acción de moderación. Sólo tiene sentido en eventos marcados: en el resto vale 0.</t>
+        </is>
+      </c>
+      <c r="C33" s="48" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="D33" s="48" t="inlineStr">
+        <is>
+          <t>minutos</t>
+        </is>
+      </c>
+      <c r="E33" s="49" t="inlineStr">
+        <is>
+          <t>En eventos marcados: mín 90,0 · p10 96,3 · mediana 140,3 · media 238,2 · p90 379,4 · máx 26.328,5. Sin las de más de 24 h: mediana 139 y p90 353</t>
+        </is>
+      </c>
+      <c r="F33" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="48" t="inlineStr">
+        <is>
+          <t>196 latencias de más de 24 h (hasta 26.328 min), que se dejan fuera. El 0 de los no marcados significa «no aplica», no «actuó al instante».</t>
+        </is>
+      </c>
+      <c r="I33" s="48" t="inlineStr">
+        <is>
+          <t>Dato. Nunca es menor que 90 min: hay un piso fijo.</t>
+        </is>
+      </c>
+      <c r="J33" s="48" t="inlineStr">
+        <is>
+          <t>Sólo existe si moderation_flag = 1. Contra la carga del momento casi no correlaciona (Spearman 0,022, el dato de D2).</t>
+        </is>
+      </c>
+      <c r="K33" s="48" t="inlineStr">
+        <is>
+          <t>Salida, no entrada: objetivo de validación. El piso de 90 min es la demora fija, y la espera por encima (mediana 49 min) calibra la escala.</t>
+        </is>
+      </c>
+      <c r="L33" s="48" t="inlineStr">
+        <is>
+          <t>D2 · D7</t>
+        </is>
+      </c>
+      <c r="M33" s="49" t="inlineStr">
+        <is>
+          <t>329,6</t>
         </is>
       </c>
     </row>
@@ -2024,7 +3337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2042,7 +3355,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Qué hacer con cada problema es parte del modelo de datos.</t>
+          <t>Qué hacer con cada problema es parte del modelo de datos. Conteos sin los duplicados, corregidos el 29/9/2026.</t>
         </is>
       </c>
     </row>
@@ -2100,7 +3413,7 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>13850</v>
+        <v>13824</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
@@ -2115,9 +3428,13 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>2008</v>
-      </c>
-      <c r="C7" s="36" t="inlineStr"/>
+        <v>2005</v>
+      </c>
+      <c r="C7" s="36" t="inlineStr">
+        <is>
+          <t>no se imputan: la columna no se usa</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2126,9 +3443,13 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>1347</v>
-      </c>
-      <c r="C8" s="36" t="inlineStr"/>
+        <v>1344</v>
+      </c>
+      <c r="C8" s="36" t="inlineStr">
+        <is>
+          <t>no se imputan: la columna no se usa</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -2137,9 +3458,13 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>1327</v>
-      </c>
-      <c r="C9" s="36" t="inlineStr"/>
+        <v>1324</v>
+      </c>
+      <c r="C9" s="36" t="inlineStr">
+        <is>
+          <t>no se imputan: la columna no se usa</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -2148,9 +3473,13 @@
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>937</v>
-      </c>
-      <c r="C10" s="36" t="inlineStr"/>
+        <v>936</v>
+      </c>
+      <c r="C10" s="36" t="inlineStr">
+        <is>
+          <t>no se imputan: la columna no se usa</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -2159,9 +3488,13 @@
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>667</v>
-      </c>
-      <c r="C11" s="36" t="inlineStr"/>
+        <v>666</v>
+      </c>
+      <c r="C11" s="36" t="inlineStr">
+        <is>
+          <t>no se imputa: el decaimiento va por generación (D18)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -2172,7 +3505,11 @@
       <c r="B12" s="16" t="n">
         <v>625</v>
       </c>
-      <c r="C12" s="36" t="inlineStr"/>
+      <c r="C12" s="36" t="inlineStr">
+        <is>
+          <t>se toman como faltantes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -2183,29 +3520,41 @@
       <c r="B13" s="16" t="n">
         <v>39</v>
       </c>
-      <c r="C13" s="36" t="inlineStr"/>
+      <c r="C13" s="36" t="inlineStr">
+        <is>
+          <t>se sacan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Hijos anteriores al padre (inter_event_time_min negativo)</t>
+          <t>inter_event_time_min negativo (las fechas de padre e hijo sí están en orden)</t>
         </is>
       </c>
       <c r="B14" s="16" t="n">
         <v>39</v>
       </c>
-      <c r="C14" s="36" t="inlineStr"/>
+      <c r="C14" s="36" t="inlineStr">
+        <is>
+          <t>se sacan del ajuste de D19</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Cuentas más viejas que la plataforma (opera desde 2013)</t>
+          <t>Eventos con antigüedad de cuenta mayor que la plataforma (opera desde 2013), de 36 cuentas</t>
         </is>
       </c>
       <c r="B15" s="16" t="n">
         <v>514</v>
       </c>
-      <c r="C15" s="36" t="inlineStr"/>
+      <c r="C15" s="36" t="inlineStr">
+        <is>
+          <t>sin efecto en ninguna estimación</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -2216,7 +3565,11 @@
       <c r="B16" s="16" t="n">
         <v>196</v>
       </c>
-      <c r="C16" s="36" t="inlineStr"/>
+      <c r="C16" s="36" t="inlineStr">
+        <is>
+          <t>se sacan</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -2227,7 +3580,11 @@
       <c r="B17" s="16" t="n">
         <v>66</v>
       </c>
-      <c r="C17" s="36" t="inlineStr"/>
+      <c r="C17" s="36" t="inlineStr">
+        <is>
+          <t>se sacan</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -2251,7 +3608,22 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>¿seguidores al momento del evento?</t>
+          <t>los seguidores se toman al momento del evento</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Hijos con fecha anterior a la del padre: son los hijos de los eventos de 2099</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>se arreglan al sacar las fechas de 2099; no es un problema aparte</t>
         </is>
       </c>
     </row>

</xml_diff>